<commit_message>
final stable bulk import fix
</commit_message>
<xml_diff>
--- a/codes.xlsx
+++ b/codes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Documents\bluerexall-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{411198B7-15E2-4491-9885-A71EEB8EBBA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B00C2E76-8E5A-4E1F-9756-9DECE5117ABC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1780" yWindow="1780" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4790,7 +4790,7 @@
   <dimension ref="A1:B1501"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.7265625" customWidth="1"/>
+    <col min="1" max="1" width="17.453125" customWidth="1"/>
     <col min="2" max="2" width="13.90625" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>